<commit_message>
Link earnings releases: first batch of the 165-model run
Partial snapshot while the full refresh-links run is in progress. Remaining
models will follow in a second commit when the run completes.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ADNH.xlsx
+++ b/ADNH.xlsx
@@ -1,150 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dillonwalton/Desktop/business/models/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ACEDE9A8-8DC0-FE48-926C-56C6449F78A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="3500" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{23AE3EDF-41AB-D84E-9A63-204D6BF85A60}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="960" yWindow="3500" windowWidth="27640" windowHeight="16940" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Main" sheetId="1" r:id="rId1"/>
-    <sheet name="Model" sheetId="2" r:id="rId2"/>
+    <sheet name="Main" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Model" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
-  <si>
-    <t>Revenue</t>
-  </si>
-  <si>
-    <t>Q120</t>
-  </si>
-  <si>
-    <t>Q220</t>
-  </si>
-  <si>
-    <t>Q320</t>
-  </si>
-  <si>
-    <t>Q420</t>
-  </si>
-  <si>
-    <t>Q121</t>
-  </si>
-  <si>
-    <t>Q221</t>
-  </si>
-  <si>
-    <t>Q321</t>
-  </si>
-  <si>
-    <t>Q422</t>
-  </si>
-  <si>
-    <t>Q421</t>
-  </si>
-  <si>
-    <t>Q122</t>
-  </si>
-  <si>
-    <t>Q222</t>
-  </si>
-  <si>
-    <t>Q322</t>
-  </si>
-  <si>
-    <t>Q123</t>
-  </si>
-  <si>
-    <t>Q223</t>
-  </si>
-  <si>
-    <t>Q323</t>
-  </si>
-  <si>
-    <t>Q423</t>
-  </si>
-  <si>
-    <t>Q124</t>
-  </si>
-  <si>
-    <t>Q224</t>
-  </si>
-  <si>
-    <t>Q324</t>
-  </si>
-  <si>
-    <t>Q424</t>
-  </si>
-  <si>
-    <t>Q125</t>
-  </si>
-  <si>
-    <t>Q225</t>
-  </si>
-  <si>
-    <t>Q325</t>
-  </si>
-  <si>
-    <t>Q425</t>
-  </si>
-  <si>
-    <t>Q126</t>
-  </si>
-  <si>
-    <t>Q226</t>
-  </si>
-  <si>
-    <t>Q326</t>
-  </si>
-  <si>
-    <t>Q426</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="FF0563C1"/>
+      <sz val="12"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -162,22 +52,82 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -608,163 +558,244 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67DDA1D6-1F4F-194C-AD5A-286704880625}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01B8BD4C-DE9E-8748-AA59-C58C6E40333D}">
-  <dimension ref="B2:AV3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:AV3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="2" spans="2:48" x14ac:dyDescent="0.2">
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N2" t="s">
-        <v>8</v>
-      </c>
-      <c r="O2" t="s">
-        <v>13</v>
-      </c>
-      <c r="P2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>15</v>
-      </c>
-      <c r="R2" t="s">
-        <v>16</v>
-      </c>
-      <c r="S2" t="s">
-        <v>17</v>
-      </c>
-      <c r="T2" t="s">
-        <v>18</v>
-      </c>
-      <c r="U2" t="s">
-        <v>19</v>
-      </c>
-      <c r="V2" t="s">
-        <v>20</v>
-      </c>
-      <c r="W2" t="s">
-        <v>21</v>
-      </c>
-      <c r="X2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>28</v>
-      </c>
-      <c r="AF2">
+    <row r="2">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Q120</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Q220</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Q320</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Q420</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Q121</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Q221</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Q321</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>Q421</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>Q122</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>Q222</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Q322</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>Q422</t>
+        </is>
+      </c>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>Q123</t>
+        </is>
+      </c>
+      <c r="P2" s="1" t="inlineStr">
+        <is>
+          <t>Q223</t>
+        </is>
+      </c>
+      <c r="Q2" s="1" t="inlineStr">
+        <is>
+          <t>Q323</t>
+        </is>
+      </c>
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>Q423</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Q124</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Q224</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Q324</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Q424</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Q125</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Q225</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Q325</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Q425</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Q126</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Q226</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Q326</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Q426</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
         <v>2020</v>
       </c>
-      <c r="AG2">
+      <c r="AG2" t="n">
         <v>2021</v>
       </c>
-      <c r="AH2">
+      <c r="AH2" t="n">
         <v>2022</v>
       </c>
-      <c r="AI2">
+      <c r="AI2" t="n">
         <v>2023</v>
       </c>
-      <c r="AJ2">
+      <c r="AJ2" t="n">
         <v>2024</v>
       </c>
-      <c r="AK2">
+      <c r="AK2" t="n">
         <v>2025</v>
       </c>
-      <c r="AL2">
+      <c r="AL2" t="n">
         <v>2026</v>
       </c>
-      <c r="AM2">
+      <c r="AM2" t="n">
         <v>2027</v>
       </c>
-      <c r="AN2">
+      <c r="AN2" t="n">
         <v>2028</v>
       </c>
-      <c r="AO2">
+      <c r="AO2" t="n">
         <v>2029</v>
       </c>
-      <c r="AP2">
+      <c r="AP2" t="n">
         <v>2030</v>
       </c>
-      <c r="AQ2">
+      <c r="AQ2" t="n">
         <v>2031</v>
       </c>
-      <c r="AR2">
+      <c r="AR2" t="n">
         <v>2032</v>
       </c>
-      <c r="AS2">
+      <c r="AS2" t="n">
         <v>2033</v>
       </c>
-      <c r="AT2">
+      <c r="AT2" t="n">
         <v>2034</v>
       </c>
-      <c r="AU2">
+      <c r="AU2" t="n">
         <v>2035</v>
       </c>
-      <c r="AV2">
+      <c r="AV2" t="n">
         <v>2036</v>
       </c>
     </row>
-    <row r="3" spans="2:48" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
-        <v>0</v>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId13"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Backfill historical links (first 41 models) and survive SEC throttling
The historical run stopped at model 41 when SEC returned 429. The abort was
correct -- blanks recorded after a throttle would be indistinguishable from
quarters that genuinely have no filing -- but a single 429 should not end a
multi-hour run.

429 is now waited out rather than fatal: honours Retry-After when present,
otherwise backs off 10s, 30s, 90s, and only gives up if throttling persists.
403 stays immediately fatal, since that is a user-agent problem rather than a
transient one.

Request interval eased from 0.11s to 0.18s (~5.5/sec). SEC publishes 10/sec,
but a sustained multi-hour run earns 429s well inside that. Overridable via
SEC_REQUEST_INTERVAL.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ADNH.xlsx
+++ b/ADNH.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -28,6 +28,13 @@
     <font>
       <name val="Aptos Narrow"/>
       <color rgb="FF0563C1"/>
+      <sz val="12"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <i val="1"/>
+      <color rgb="FF7030A0"/>
       <sz val="12"/>
       <u val="single"/>
     </font>
@@ -52,9 +59,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -576,47 +584,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC3"/>
+  <dimension ref="A2:BC3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Q418</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Q119</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Q219</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Q319</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Q419</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Q120</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Q220</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Q320</t>
         </is>
@@ -686,37 +693,37 @@
           <t>Q423</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>Q124</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>Q224</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>Q324</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>Q424</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>Q125</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>Q225</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AD2" s="2" t="inlineStr">
         <is>
           <t>Q325</t>
         </is>
@@ -813,21 +820,36 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T2" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V2" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T2" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V2" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y2" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z2" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
 </worksheet>
 </file>
</xml_diff>